<commit_message>
Fix missing calculation on calculate row 14 (roster_index)
</commit_message>
<xml_diff>
--- a/forms/reference-form.xlsx
+++ b/forms/reference-form.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\Survey\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faith\FaithWambui\Cross Platform Survey Toolkit\forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7461D31F-9015-4D0B-B891-FA437D9B43EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DEA6DBD-0E92-4F67-995E-21CFB04088CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" activeTab="2" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="11866" windowHeight="14963" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -4633,7 +4633,7 @@
       <c r="B14" t="s">
         <v>1131</v>
       </c>
-      <c r="F14" t="s">
+      <c r="I14" t="s">
         <v>1132</v>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>1140</v>
       </c>
@@ -4694,7 +4694,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>1146</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>1150</v>
       </c>
@@ -4728,7 +4728,7 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>1155</v>
       </c>
@@ -4745,7 +4745,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>1160</v>
       </c>
@@ -4762,7 +4762,7 @@
         <v>1164</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -4813,7 +4813,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -4830,7 +4830,7 @@
         <v>1177</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>1178</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>24</v>
       </c>
@@ -4878,7 +4878,7 @@
         <v>1188</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>1189</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>1126</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>1130</v>
       </c>
@@ -4896,11 +4896,11 @@
       <c r="C30" t="s">
         <v>1191</v>
       </c>
-      <c r="G30" t="s">
+      <c r="I30" t="s">
         <v>1192</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>1193</v>
       </c>
@@ -4926,7 +4926,7 @@
         <v>1198</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>1193</v>
       </c>
@@ -4988,7 +4988,7 @@
       <c r="C34" t="s">
         <v>1209</v>
       </c>
-      <c r="G34" t="s">
+      <c r="I34" t="s">
         <v>1210</v>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
         <v>1261</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>1140</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>1261</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>1140</v>
       </c>
@@ -5336,7 +5336,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>1272</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>37</v>
       </c>
@@ -5373,7 +5373,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>1178</v>
       </c>
@@ -5390,7 +5390,7 @@
         <v>1282</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>1283</v>
       </c>
@@ -5410,7 +5410,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>1140</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>1140</v>
       </c>
@@ -5462,7 +5462,7 @@
         <v>1296</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>37</v>
       </c>
@@ -5482,7 +5482,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>1300</v>
       </c>
@@ -5499,7 +5499,7 @@
         <v>1303</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>37</v>
       </c>
@@ -5519,7 +5519,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>37</v>
       </c>
@@ -5539,7 +5539,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>1310</v>
       </c>
@@ -5556,7 +5556,7 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>24</v>
       </c>
@@ -5573,7 +5573,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>1130</v>
       </c>
@@ -5583,11 +5583,11 @@
       <c r="C63" t="s">
         <v>1319</v>
       </c>
-      <c r="G63" t="s">
+      <c r="I63" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>1272</v>
       </c>

</xml_diff>

<commit_message>
Add relevant logic for cascading geography titles and update translation notes
</commit_message>
<xml_diff>
--- a/forms/reference-form.xlsx
+++ b/forms/reference-form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faith\FaithWambui\Cross Platform Survey Toolkit\forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DEA6DBD-0E92-4F67-995E-21CFB04088CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769D1622-6178-4D5C-8C86-A2522A4F5F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-83" yWindow="0" windowWidth="11866" windowHeight="14963" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
   </bookViews>
@@ -3377,18 +3377,12 @@
     <t>Chagua Kaunti</t>
   </si>
   <si>
-    <t>choice_filter: region=${region}</t>
-  </si>
-  <si>
     <t>Select Sub-County</t>
   </si>
   <si>
     <t>Chagua Kaunti Ndogo</t>
   </si>
   <si>
-    <t>choice_filter: county=${county}</t>
-  </si>
-  <si>
     <t>Nambari ya Kaya</t>
   </si>
   <si>
@@ -4029,6 +4023,12 @@
   </si>
   <si>
     <t>KES 30,000 - 49,999</t>
+  </si>
+  <si>
+    <t>region=${region}</t>
+  </si>
+  <si>
+    <t>county=${county}</t>
   </si>
 </sst>
 </file>
@@ -4534,8 +4534,8 @@
       <c r="E8" t="s">
         <v>31</v>
       </c>
-      <c r="K8" t="s">
-        <v>1116</v>
+      <c r="J8" t="s">
+        <v>1332</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
@@ -4546,16 +4546,16 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D9" t="s">
         <v>1117</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1118</v>
       </c>
       <c r="E9" t="s">
         <v>31</v>
       </c>
-      <c r="K9" t="s">
-        <v>1119</v>
+      <c r="J9" t="s">
+        <v>1333</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.45">
@@ -4569,7 +4569,7 @@
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="E10" t="s">
         <v>31</v>
@@ -4583,10 +4583,10 @@
         <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="D11" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="E11" t="s">
         <v>31</v>
@@ -4600,10 +4600,10 @@
         <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="D12" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="E12" t="s">
         <v>31</v>
@@ -4611,30 +4611,30 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C13" t="s">
         <v>1125</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
         <v>1126</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
         <v>1127</v>
-      </c>
-      <c r="D13" t="s">
-        <v>1128</v>
-      </c>
-      <c r="F13" t="s">
-        <v>1129</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1129</v>
+      </c>
+      <c r="I14" t="s">
         <v>1130</v>
-      </c>
-      <c r="B14" t="s">
-        <v>1131</v>
-      </c>
-      <c r="I14" t="s">
-        <v>1132</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.45">
@@ -4642,13 +4642,13 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1132</v>
+      </c>
+      <c r="D15" t="s">
         <v>1133</v>
-      </c>
-      <c r="C15" t="s">
-        <v>1134</v>
-      </c>
-      <c r="D15" t="s">
-        <v>1135</v>
       </c>
       <c r="E15" t="s">
         <v>31</v>
@@ -4656,16 +4656,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C16" t="s">
         <v>1136</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>1137</v>
-      </c>
-      <c r="C16" t="s">
-        <v>1138</v>
-      </c>
-      <c r="D16" t="s">
-        <v>1139</v>
       </c>
       <c r="E16" t="s">
         <v>31</v>
@@ -4673,39 +4673,39 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C17" t="s">
         <v>1140</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
         <v>1141</v>
-      </c>
-      <c r="C17" t="s">
-        <v>1142</v>
-      </c>
-      <c r="D17" t="s">
-        <v>1143</v>
       </c>
       <c r="E17" t="s">
         <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="H17" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
+        <v>1144</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C18" t="s">
         <v>1146</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>1147</v>
-      </c>
-      <c r="C18" t="s">
-        <v>1148</v>
-      </c>
-      <c r="D18" t="s">
-        <v>1149</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
@@ -4713,53 +4713,53 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C19" t="s">
         <v>1150</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
         <v>1151</v>
       </c>
-      <c r="C19" t="s">
+      <c r="F19" t="s">
         <v>1152</v>
-      </c>
-      <c r="D19" t="s">
-        <v>1153</v>
-      </c>
-      <c r="F19" t="s">
-        <v>1154</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C20" t="s">
         <v>1155</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>1156</v>
       </c>
-      <c r="C20" t="s">
+      <c r="F20" t="s">
         <v>1157</v>
-      </c>
-      <c r="D20" t="s">
-        <v>1158</v>
-      </c>
-      <c r="F20" t="s">
-        <v>1159</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C21" t="s">
         <v>1160</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>1161</v>
       </c>
-      <c r="C21" t="s">
+      <c r="F21" t="s">
         <v>1162</v>
-      </c>
-      <c r="D21" t="s">
-        <v>1163</v>
-      </c>
-      <c r="F21" t="s">
-        <v>1164</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.45">
@@ -4767,13 +4767,13 @@
         <v>37</v>
       </c>
       <c r="B22" t="s">
+        <v>1163</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D22" t="s">
         <v>1165</v>
-      </c>
-      <c r="C22" t="s">
-        <v>1166</v>
-      </c>
-      <c r="D22" t="s">
-        <v>1167</v>
       </c>
       <c r="E22" t="s">
         <v>31</v>
@@ -4784,13 +4784,13 @@
         <v>37</v>
       </c>
       <c r="B23" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D23" t="s">
         <v>1168</v>
-      </c>
-      <c r="C23" t="s">
-        <v>1169</v>
-      </c>
-      <c r="D23" t="s">
-        <v>1170</v>
       </c>
       <c r="E23" t="s">
         <v>31</v>
@@ -4801,16 +4801,16 @@
         <v>37</v>
       </c>
       <c r="B24" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D24" t="s">
         <v>1171</v>
       </c>
-      <c r="C24" t="s">
-        <v>1172</v>
-      </c>
-      <c r="D24" t="s">
-        <v>1173</v>
-      </c>
       <c r="F24" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.45">
@@ -4818,33 +4818,33 @@
         <v>37</v>
       </c>
       <c r="B25" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1173</v>
+      </c>
+      <c r="D25" t="s">
         <v>1174</v>
       </c>
-      <c r="C25" t="s">
+      <c r="F25" t="s">
         <v>1175</v>
-      </c>
-      <c r="D25" t="s">
-        <v>1176</v>
-      </c>
-      <c r="F25" t="s">
-        <v>1177</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C26" t="s">
         <v>1178</v>
       </c>
-      <c r="B26" t="s">
+      <c r="D26" t="s">
         <v>1179</v>
       </c>
-      <c r="C26" t="s">
+      <c r="F26" t="s">
         <v>1180</v>
-      </c>
-      <c r="D26" t="s">
-        <v>1181</v>
-      </c>
-      <c r="F26" t="s">
-        <v>1182</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.45">
@@ -4852,13 +4852,13 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1182</v>
+      </c>
+      <c r="D27" t="s">
         <v>1183</v>
-      </c>
-      <c r="C27" t="s">
-        <v>1184</v>
-      </c>
-      <c r="D27" t="s">
-        <v>1185</v>
       </c>
       <c r="E27" t="s">
         <v>31</v>
@@ -4869,488 +4869,488 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D28" t="s">
         <v>1186</v>
-      </c>
-      <c r="C28" t="s">
-        <v>1187</v>
-      </c>
-      <c r="D28" t="s">
-        <v>1188</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="B29" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="B30" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1189</v>
+      </c>
+      <c r="I30" t="s">
         <v>1190</v>
-      </c>
-      <c r="C30" t="s">
-        <v>1191</v>
-      </c>
-      <c r="I30" t="s">
-        <v>1192</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C31" t="s">
         <v>1193</v>
       </c>
-      <c r="B31" t="s">
+      <c r="D31" t="s">
         <v>1194</v>
-      </c>
-      <c r="C31" t="s">
-        <v>1195</v>
-      </c>
-      <c r="D31" t="s">
-        <v>1196</v>
       </c>
       <c r="E31" t="s">
         <v>31</v>
       </c>
       <c r="F31" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G31" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="H31" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="B32" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1198</v>
+      </c>
+      <c r="D32" t="s">
         <v>1199</v>
-      </c>
-      <c r="C32" t="s">
-        <v>1200</v>
-      </c>
-      <c r="D32" t="s">
-        <v>1201</v>
       </c>
       <c r="E32" t="s">
         <v>31</v>
       </c>
       <c r="F32" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G32" t="s">
+        <v>1200</v>
+      </c>
+      <c r="H32" t="s">
+        <v>1201</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B33" t="s">
         <v>1202</v>
       </c>
-      <c r="H32" t="s">
+      <c r="C33" t="s">
         <v>1203</v>
       </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>1193</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="D33" t="s">
         <v>1204</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1205</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1206</v>
       </c>
       <c r="E33" t="s">
         <v>31</v>
       </c>
       <c r="F33" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G33" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="H33" t="s">
+        <v>1205</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1206</v>
+      </c>
+      <c r="C34" t="s">
         <v>1207</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
-        <v>1130</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="I34" t="s">
         <v>1208</v>
       </c>
-      <c r="C34" t="s">
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
         <v>1209</v>
       </c>
-      <c r="I34" t="s">
+      <c r="B35" t="s">
         <v>1210</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+      <c r="C35" t="s">
         <v>1211</v>
       </c>
-      <c r="B35" t="s">
+      <c r="D35" t="s">
         <v>1212</v>
-      </c>
-      <c r="C35" t="s">
-        <v>1213</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1214</v>
       </c>
       <c r="E35" t="s">
         <v>31</v>
       </c>
       <c r="F35" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>37</v>
       </c>
       <c r="B36" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1214</v>
+      </c>
+      <c r="D36" t="s">
         <v>1215</v>
       </c>
-      <c r="C36" t="s">
+      <c r="F36" t="s">
         <v>1216</v>
       </c>
-      <c r="D36" t="s">
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B37" t="s">
         <v>1217</v>
       </c>
-      <c r="F36" t="s">
+      <c r="C37" t="s">
         <v>1218</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>1193</v>
-      </c>
-      <c r="B37" t="s">
+      <c r="D37" t="s">
         <v>1219</v>
       </c>
-      <c r="C37" t="s">
+      <c r="F37" t="s">
         <v>1220</v>
       </c>
-      <c r="D37" t="s">
+      <c r="G37" t="s">
         <v>1221</v>
       </c>
-      <c r="F37" t="s">
+      <c r="H37" t="s">
         <v>1222</v>
       </c>
-      <c r="G37" t="s">
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
         <v>1223</v>
       </c>
-      <c r="H37" t="s">
+      <c r="B38" t="s">
         <v>1224</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
+      <c r="C38" t="s">
         <v>1225</v>
       </c>
-      <c r="B38" t="s">
+      <c r="D38" t="s">
         <v>1226</v>
-      </c>
-      <c r="C38" t="s">
-        <v>1227</v>
-      </c>
-      <c r="D38" t="s">
-        <v>1228</v>
       </c>
       <c r="E38" t="s">
         <v>31</v>
       </c>
       <c r="F38" t="s">
-        <v>1129</v>
-      </c>
-      <c r="L38" t="s">
-        <v>1119</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+      <c r="J38" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>1225</v>
+        <v>1223</v>
       </c>
       <c r="B39" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D39" t="s">
         <v>1229</v>
-      </c>
-      <c r="C39" t="s">
-        <v>1230</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1231</v>
       </c>
       <c r="E39" t="s">
         <v>31</v>
       </c>
       <c r="F39" t="s">
-        <v>1129</v>
-      </c>
-      <c r="L39" t="s">
-        <v>1119</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+      <c r="J39" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>1225</v>
+        <v>1223</v>
       </c>
       <c r="B40" t="s">
+        <v>1230</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1231</v>
+      </c>
+      <c r="D40" t="s">
         <v>1232</v>
       </c>
-      <c r="C40" t="s">
+      <c r="F40" t="s">
+        <v>1127</v>
+      </c>
+      <c r="J40" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B41" t="s">
         <v>1233</v>
       </c>
-      <c r="D40" t="s">
+      <c r="C41" t="s">
         <v>1234</v>
       </c>
-      <c r="F40" t="s">
-        <v>1129</v>
-      </c>
-      <c r="L40" t="s">
-        <v>1119</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
-        <v>1193</v>
-      </c>
-      <c r="B41" t="s">
+      <c r="D41" t="s">
         <v>1235</v>
-      </c>
-      <c r="C41" t="s">
-        <v>1236</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1237</v>
       </c>
       <c r="E41" t="s">
         <v>31</v>
       </c>
       <c r="F41" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G41" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="H41" t="s">
-        <v>1238</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>37</v>
       </c>
       <c r="B42" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1238</v>
+      </c>
+      <c r="D42" t="s">
         <v>1239</v>
-      </c>
-      <c r="C42" t="s">
-        <v>1240</v>
-      </c>
-      <c r="D42" t="s">
-        <v>1241</v>
       </c>
       <c r="E42" t="s">
         <v>31</v>
       </c>
       <c r="F42" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C43" t="s">
         <v>1242</v>
       </c>
-      <c r="B43" t="s">
+      <c r="D43" t="s">
         <v>1243</v>
       </c>
-      <c r="C43" t="s">
+      <c r="F43" t="s">
         <v>1244</v>
       </c>
-      <c r="D43" t="s">
-        <v>1245</v>
-      </c>
-      <c r="F43" t="s">
-        <v>1246</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.45">
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>37</v>
       </c>
       <c r="B44" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1246</v>
+      </c>
+      <c r="D44" t="s">
         <v>1247</v>
-      </c>
-      <c r="C44" t="s">
-        <v>1248</v>
-      </c>
-      <c r="D44" t="s">
-        <v>1249</v>
       </c>
       <c r="E44" t="s">
         <v>31</v>
       </c>
       <c r="F44" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>37</v>
       </c>
       <c r="B45" t="s">
+        <v>1248</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D45" t="s">
         <v>1250</v>
-      </c>
-      <c r="C45" t="s">
-        <v>1251</v>
-      </c>
-      <c r="D45" t="s">
-        <v>1252</v>
       </c>
       <c r="E45" t="s">
         <v>31</v>
       </c>
       <c r="F45" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>37</v>
       </c>
       <c r="B46" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D46" t="s">
         <v>1253</v>
-      </c>
-      <c r="C46" t="s">
-        <v>1254</v>
-      </c>
-      <c r="D46" t="s">
-        <v>1255</v>
       </c>
       <c r="E46" t="s">
         <v>31</v>
       </c>
       <c r="F46" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.45">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="B47" t="s">
+        <v>1254</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1255</v>
+      </c>
+      <c r="D47" t="s">
         <v>1256</v>
       </c>
-      <c r="C47" t="s">
+      <c r="F47" t="s">
         <v>1257</v>
       </c>
-      <c r="D47" t="s">
+      <c r="G47" t="s">
         <v>1258</v>
       </c>
-      <c r="F47" t="s">
+      <c r="H47" t="s">
         <v>1259</v>
       </c>
-      <c r="G47" t="s">
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B48" t="s">
         <v>1260</v>
       </c>
-      <c r="H47" t="s">
+      <c r="C48" t="s">
         <v>1261</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
-        <v>1140</v>
-      </c>
-      <c r="B48" t="s">
+      <c r="D48" t="s">
         <v>1262</v>
       </c>
-      <c r="C48" t="s">
-        <v>1263</v>
-      </c>
-      <c r="D48" t="s">
-        <v>1264</v>
-      </c>
       <c r="F48" t="s">
+        <v>1257</v>
+      </c>
+      <c r="G48" t="s">
+        <v>1258</v>
+      </c>
+      <c r="H48" t="s">
         <v>1259</v>
-      </c>
-      <c r="G48" t="s">
-        <v>1260</v>
-      </c>
-      <c r="H48" t="s">
-        <v>1261</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="B49" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D49" t="s">
         <v>1265</v>
       </c>
-      <c r="C49" t="s">
-        <v>1266</v>
-      </c>
-      <c r="D49" t="s">
-        <v>1267</v>
-      </c>
       <c r="F49" t="s">
+        <v>1257</v>
+      </c>
+      <c r="G49" t="s">
+        <v>1258</v>
+      </c>
+      <c r="H49" t="s">
         <v>1259</v>
-      </c>
-      <c r="G49" t="s">
-        <v>1260</v>
-      </c>
-      <c r="H49" t="s">
-        <v>1261</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="B50" t="s">
+        <v>1266</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1267</v>
+      </c>
+      <c r="D50" t="s">
         <v>1268</v>
-      </c>
-      <c r="C50" t="s">
-        <v>1269</v>
-      </c>
-      <c r="D50" t="s">
-        <v>1270</v>
       </c>
       <c r="E50" t="s">
         <v>31</v>
       </c>
       <c r="F50" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G50" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
       <c r="H50" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B51" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C51" t="s">
         <v>1272</v>
       </c>
-      <c r="B51" t="s">
+      <c r="D51" t="s">
         <v>1273</v>
       </c>
-      <c r="C51" t="s">
-        <v>1274</v>
-      </c>
-      <c r="D51" t="s">
-        <v>1275</v>
-      </c>
       <c r="F51" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.45">
@@ -5358,108 +5358,108 @@
         <v>37</v>
       </c>
       <c r="B52" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1275</v>
+      </c>
+      <c r="D52" t="s">
         <v>1276</v>
-      </c>
-      <c r="C52" t="s">
-        <v>1277</v>
-      </c>
-      <c r="D52" t="s">
-        <v>1278</v>
       </c>
       <c r="E52" t="s">
         <v>31</v>
       </c>
       <c r="F52" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="B53" t="s">
+        <v>1277</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1278</v>
+      </c>
+      <c r="D53" t="s">
         <v>1279</v>
       </c>
-      <c r="C53" t="s">
+      <c r="F53" t="s">
         <v>1280</v>
-      </c>
-      <c r="D53" t="s">
-        <v>1281</v>
-      </c>
-      <c r="F53" t="s">
-        <v>1282</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C54" t="s">
         <v>1283</v>
       </c>
-      <c r="B54" t="s">
+      <c r="D54" t="s">
         <v>1284</v>
-      </c>
-      <c r="C54" t="s">
-        <v>1285</v>
-      </c>
-      <c r="D54" t="s">
-        <v>1286</v>
       </c>
       <c r="E54" t="s">
         <v>31</v>
       </c>
       <c r="F54" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="B55" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1286</v>
+      </c>
+      <c r="D55" t="s">
         <v>1287</v>
-      </c>
-      <c r="C55" t="s">
-        <v>1288</v>
-      </c>
-      <c r="D55" t="s">
-        <v>1289</v>
       </c>
       <c r="E55" t="s">
         <v>31</v>
       </c>
       <c r="F55" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G55" t="s">
-        <v>1290</v>
+        <v>1288</v>
       </c>
       <c r="H55" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="B56" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D56" t="s">
         <v>1292</v>
-      </c>
-      <c r="C56" t="s">
-        <v>1293</v>
-      </c>
-      <c r="D56" t="s">
-        <v>1294</v>
       </c>
       <c r="E56" t="s">
         <v>31</v>
       </c>
       <c r="F56" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G56" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
       <c r="H56" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.45">
@@ -5467,36 +5467,36 @@
         <v>37</v>
       </c>
       <c r="B57" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1296</v>
+      </c>
+      <c r="D57" t="s">
         <v>1297</v>
-      </c>
-      <c r="C57" t="s">
-        <v>1298</v>
-      </c>
-      <c r="D57" t="s">
-        <v>1299</v>
       </c>
       <c r="E57" t="s">
         <v>31</v>
       </c>
       <c r="F57" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
       <c r="B58" t="s">
         <v>1065</v>
       </c>
       <c r="C58" t="s">
+        <v>1299</v>
+      </c>
+      <c r="D58" t="s">
+        <v>1300</v>
+      </c>
+      <c r="F58" t="s">
         <v>1301</v>
-      </c>
-      <c r="D58" t="s">
-        <v>1302</v>
-      </c>
-      <c r="F58" t="s">
-        <v>1303</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.45">
@@ -5504,19 +5504,19 @@
         <v>37</v>
       </c>
       <c r="B59" t="s">
+        <v>1302</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1303</v>
+      </c>
+      <c r="D59" t="s">
         <v>1304</v>
-      </c>
-      <c r="C59" t="s">
-        <v>1305</v>
-      </c>
-      <c r="D59" t="s">
-        <v>1306</v>
       </c>
       <c r="E59" t="s">
         <v>31</v>
       </c>
       <c r="F59" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.45">
@@ -5524,36 +5524,36 @@
         <v>37</v>
       </c>
       <c r="B60" t="s">
+        <v>1305</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1306</v>
+      </c>
+      <c r="D60" t="s">
         <v>1307</v>
-      </c>
-      <c r="C60" t="s">
-        <v>1308</v>
-      </c>
-      <c r="D60" t="s">
-        <v>1309</v>
       </c>
       <c r="E60" t="s">
         <v>31</v>
       </c>
       <c r="F60" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B61" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C61" t="s">
         <v>1310</v>
       </c>
-      <c r="B61" t="s">
+      <c r="D61" t="s">
         <v>1311</v>
       </c>
-      <c r="C61" t="s">
+      <c r="F61" t="s">
         <v>1312</v>
-      </c>
-      <c r="D61" t="s">
-        <v>1313</v>
-      </c>
-      <c r="F61" t="s">
-        <v>1314</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.45">
@@ -5561,70 +5561,70 @@
         <v>24</v>
       </c>
       <c r="B62" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C62" t="s">
+        <v>1314</v>
+      </c>
+      <c r="D62" t="s">
         <v>1315</v>
       </c>
-      <c r="C62" t="s">
-        <v>1316</v>
-      </c>
-      <c r="D62" t="s">
-        <v>1317</v>
-      </c>
       <c r="F62" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="B63" t="s">
+        <v>1316</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1317</v>
+      </c>
+      <c r="I63" t="s">
         <v>1318</v>
-      </c>
-      <c r="C63" t="s">
-        <v>1319</v>
-      </c>
-      <c r="I63" t="s">
-        <v>1320</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
       <c r="B64" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1320</v>
+      </c>
+      <c r="D64" t="s">
         <v>1321</v>
       </c>
-      <c r="C64" t="s">
-        <v>1322</v>
-      </c>
-      <c r="D64" t="s">
-        <v>1323</v>
-      </c>
       <c r="F64" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
       <c r="B65" t="s">
+        <v>1322</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1323</v>
+      </c>
+      <c r="D65" t="s">
         <v>1324</v>
-      </c>
-      <c r="C65" t="s">
-        <v>1325</v>
-      </c>
-      <c r="D65" t="s">
-        <v>1326</v>
       </c>
       <c r="E65" t="s">
         <v>31</v>
       </c>
       <c r="F65" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="L65" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
     </row>
   </sheetData>
@@ -12577,10 +12577,10 @@
         <v>1059</v>
       </c>
       <c r="C421" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
       <c r="D421" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.45">
@@ -12591,10 +12591,10 @@
         <v>1060</v>
       </c>
       <c r="C422" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="D422" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.45">
@@ -12605,10 +12605,10 @@
         <v>1061</v>
       </c>
       <c r="C423" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="D423" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Complete SurveyCTO deployment verification and update translation notes
</commit_message>
<xml_diff>
--- a/forms/reference-form.xlsx
+++ b/forms/reference-form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faith\FaithWambui\Cross Platform Survey Toolkit\forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{769D1622-6178-4D5C-8C86-A2522A4F5F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4813EC60-4D65-4B86-B102-27C2AB2A45EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="11866" windowHeight="14963" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
+    <workbookView xWindow="11617" yWindow="0" windowWidth="11865" windowHeight="14963" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="1334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2474" uniqueCount="1336">
   <si>
     <t>type</t>
   </si>
@@ -4029,6 +4029,12 @@
   </si>
   <si>
     <t>county=${county}</t>
+  </si>
+  <si>
+    <t>${region} != ''</t>
+  </si>
+  <si>
+    <t>${county} != ''</t>
   </si>
 </sst>
 </file>
@@ -4534,6 +4540,9 @@
       <c r="E8" t="s">
         <v>31</v>
       </c>
+      <c r="F8" t="s">
+        <v>1334</v>
+      </c>
       <c r="J8" t="s">
         <v>1332</v>
       </c>
@@ -4554,6 +4563,9 @@
       <c r="E9" t="s">
         <v>31</v>
       </c>
+      <c r="F9" t="s">
+        <v>1335</v>
+      </c>
       <c r="J9" t="s">
         <v>1333</v>
       </c>
@@ -4952,7 +4964,7 @@
         <v>1201</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>1191</v>
       </c>
@@ -4978,7 +4990,7 @@
         <v>1205</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>1128</v>
       </c>
@@ -4992,7 +5004,7 @@
         <v>1208</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>1209</v>
       </c>
@@ -5012,7 +5024,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -5029,7 +5041,7 @@
         <v>1216</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>1191</v>
       </c>
@@ -5052,7 +5064,7 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>1223</v>
       </c>
@@ -5071,11 +5083,8 @@
       <c r="F38" t="s">
         <v>1127</v>
       </c>
-      <c r="J38" t="s">
-        <v>1333</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>1223</v>
       </c>
@@ -5094,11 +5103,8 @@
       <c r="F39" t="s">
         <v>1127</v>
       </c>
-      <c r="J39" t="s">
-        <v>1333</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>1223</v>
       </c>
@@ -5114,11 +5120,8 @@
       <c r="F40" t="s">
         <v>1127</v>
       </c>
-      <c r="J40" t="s">
-        <v>1333</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>1191</v>
       </c>
@@ -5144,7 +5147,7 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>37</v>
       </c>
@@ -5164,7 +5167,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>1240</v>
       </c>
@@ -5181,7 +5184,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>37</v>
       </c>
@@ -5201,7 +5204,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>37</v>
       </c>
@@ -5221,7 +5224,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>37</v>
       </c>
@@ -5241,7 +5244,7 @@
         <v>1127</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>1138</v>
       </c>
@@ -5264,7 +5267,7 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>1138</v>
       </c>
@@ -5327,7 +5330,7 @@
         <v>31</v>
       </c>
       <c r="F50" t="s">
-        <v>1127</v>
+        <v>1257</v>
       </c>
       <c r="G50" t="s">
         <v>1258</v>

</xml_diff>

<commit_message>
Update master reference-form.xlsx with livestock group skip logic
</commit_message>
<xml_diff>
--- a/forms/reference-form.xlsx
+++ b/forms/reference-form.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faith\FaithWambui\Cross Platform Survey Toolkit\forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4813EC60-4D65-4B86-B102-27C2AB2A45EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63AFE8C1-0721-4378-A855-DF079BFBCA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11617" yWindow="0" windowWidth="11865" windowHeight="14963" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
+    <workbookView xWindow="11617" yWindow="0" windowWidth="11865" windowHeight="14963" activeTab="1" xr2:uid="{3883F40F-EC26-4374-8A14-C8E6FA28D05D}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>

</xml_diff>